<commit_message>
fix: 원천 데이터 필드명 전체 경로로 수정 (l_sap.orderlist.vf219/vf599)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/efficiency_profit_dev_request.xlsx
+++ b/efficiency_profit_dev_request.xlsx
@@ -877,7 +877,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>vf219</t>
+          <t>l_sap.orderlist.vf219</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>상품 코드 · 연도 기준 컬럼 — 개발팀 확인 필요</t>
+          <t>상품 코드 · 연도 기준 컬럼 — SDSC 확인 필요</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>vf599</t>
+          <t>l_sap.orderlist.vf599</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>상품 코드 · 연도 기준 컬럼 — 개발팀 확인 필요</t>
+          <t>상품 코드 · 연도 기준 컬럼 — SDSC 확인 필요</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>개발팀 확인 필요</t>
+          <t>SDSC 확인 필요</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">

</xml_diff>